<commit_message>
Refresh E2E evidence screenshots after go-live regression sweep
Full 17-suite Playwright run (311/311 checks) against the Sales Report
Summary fix and the import-preview clarification, confirming no
regressions before deploy.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T4LurPsVU5WNa1i8str9pz
</commit_message>
<xml_diff>
--- a/e2e-screenshots/batch-vs-marketplace/downloaded-inventory-report.xlsx
+++ b/e2e-screenshots/batch-vs-marketplace/downloaded-inventory-report.xlsx
@@ -818,7 +818,7 @@
         <v>21</v>
       </c>
       <c r="L2">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -856,7 +856,7 @@
         <v>21</v>
       </c>
       <c r="L3">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -894,7 +894,7 @@
         <v>21</v>
       </c>
       <c r="L4">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -932,7 +932,7 @@
         <v>21</v>
       </c>
       <c r="L5">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -970,7 +970,7 @@
         <v>21</v>
       </c>
       <c r="L6">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -1008,7 +1008,7 @@
         <v>21</v>
       </c>
       <c r="L7">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -1046,7 +1046,7 @@
         <v>21</v>
       </c>
       <c r="L8">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
@@ -1084,7 +1084,7 @@
         <v>21</v>
       </c>
       <c r="L9">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
@@ -1122,7 +1122,7 @@
         <v>21</v>
       </c>
       <c r="L10">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
@@ -1160,7 +1160,7 @@
         <v>21</v>
       </c>
       <c r="L11">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
@@ -1198,7 +1198,7 @@
         <v>21</v>
       </c>
       <c r="L12">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
@@ -1236,7 +1236,7 @@
         <v>21</v>
       </c>
       <c r="L13">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
@@ -1274,7 +1274,7 @@
         <v>21</v>
       </c>
       <c r="L14">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
@@ -1312,7 +1312,7 @@
         <v>21</v>
       </c>
       <c r="L15">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
@@ -1350,7 +1350,7 @@
         <v>21</v>
       </c>
       <c r="L16">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
@@ -1388,7 +1388,7 @@
         <v>21</v>
       </c>
       <c r="L17">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
@@ -1426,7 +1426,7 @@
         <v>21</v>
       </c>
       <c r="L18">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
@@ -1464,7 +1464,7 @@
         <v>21</v>
       </c>
       <c r="L19">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
@@ -1502,7 +1502,7 @@
         <v>21</v>
       </c>
       <c r="L20">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
@@ -1540,7 +1540,7 @@
         <v>21</v>
       </c>
       <c r="L21">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
@@ -1578,7 +1578,7 @@
         <v>21</v>
       </c>
       <c r="L22">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
@@ -1616,7 +1616,7 @@
         <v>21</v>
       </c>
       <c r="L23">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
@@ -1654,7 +1654,7 @@
         <v>21</v>
       </c>
       <c r="L24">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
@@ -1692,7 +1692,7 @@
         <v>21</v>
       </c>
       <c r="L25">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
@@ -1730,7 +1730,7 @@
         <v>21</v>
       </c>
       <c r="L26">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
@@ -1768,7 +1768,7 @@
         <v>21</v>
       </c>
       <c r="L27">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
@@ -1806,7 +1806,7 @@
         <v>21</v>
       </c>
       <c r="L28">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
@@ -1844,7 +1844,7 @@
         <v>21</v>
       </c>
       <c r="L29">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -1939,7 +1939,7 @@
         <v>102</v>
       </c>
       <c r="L2">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -1977,7 +1977,7 @@
         <v>102</v>
       </c>
       <c r="L3">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -2015,7 +2015,7 @@
         <v>102</v>
       </c>
       <c r="L4">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -2053,7 +2053,7 @@
         <v>102</v>
       </c>
       <c r="L5">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -2091,7 +2091,7 @@
         <v>102</v>
       </c>
       <c r="L6">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -2129,7 +2129,7 @@
         <v>102</v>
       </c>
       <c r="L7">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -2167,7 +2167,7 @@
         <v>102</v>
       </c>
       <c r="L8">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
@@ -2205,7 +2205,7 @@
         <v>102</v>
       </c>
       <c r="L9">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
@@ -2243,7 +2243,7 @@
         <v>102</v>
       </c>
       <c r="L10">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
@@ -2281,7 +2281,7 @@
         <v>102</v>
       </c>
       <c r="L11">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh e2e artifacts from the running sweep
Screenshots and downloaded workbooks regenerated by the re-runs.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T4LurPsVU5WNa1i8str9pz
</commit_message>
<xml_diff>
--- a/e2e-screenshots/batch-vs-marketplace/downloaded-inventory-report.xlsx
+++ b/e2e-screenshots/batch-vs-marketplace/downloaded-inventory-report.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="110">
   <si>
     <t>Stock In Date</t>
   </si>
@@ -48,6 +48,9 @@
   </si>
   <si>
     <t>Age (days)</t>
+  </si>
+  <si>
+    <t>Return Date</t>
   </si>
   <si>
     <t>2026-07-20</t>
@@ -735,17 +738,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:M29"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="10" width="14" customWidth="1"/>
     <col min="11" max="11" width="30" customWidth="1"/>
-    <col min="12" max="12" width="14" customWidth="1"/>
+    <col min="12" max="13" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -782,1073 +785,1160 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I2">
         <v>517.1</v>
       </c>
       <c r="J2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L2">
+        <v>51</v>
+      </c>
+      <c r="M2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F3" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" t="s">
-        <v>17</v>
-      </c>
       <c r="G3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I3">
         <v>327.58</v>
       </c>
       <c r="J3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L3">
+        <v>52</v>
+      </c>
+      <c r="M3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H4" t="s">
         <v>20</v>
-      </c>
-      <c r="K3" t="s">
-        <v>21</v>
-      </c>
-      <c r="L3">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D4" t="s">
-        <v>30</v>
-      </c>
-      <c r="E4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G4" t="s">
-        <v>32</v>
-      </c>
-      <c r="H4" t="s">
-        <v>19</v>
       </c>
       <c r="I4">
         <v>223.04</v>
       </c>
       <c r="J4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+      <c r="M4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I5">
         <v>293.74</v>
       </c>
       <c r="J5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L5">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+      <c r="M5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" t="s">
+        <v>42</v>
+      </c>
+      <c r="D6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" t="s">
+        <v>43</v>
+      </c>
+      <c r="H6" t="s">
         <v>39</v>
-      </c>
-      <c r="B6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C6" t="s">
-        <v>41</v>
-      </c>
-      <c r="D6" t="s">
-        <v>36</v>
-      </c>
-      <c r="E6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F6" t="s">
-        <v>17</v>
-      </c>
-      <c r="G6" t="s">
-        <v>42</v>
-      </c>
-      <c r="H6" t="s">
-        <v>38</v>
       </c>
       <c r="I6">
         <v>417.16</v>
       </c>
       <c r="J6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L6">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+      <c r="M6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I7">
         <v>242</v>
       </c>
       <c r="J7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K7" t="s">
+        <v>22</v>
+      </c>
+      <c r="L7">
+        <v>57</v>
+      </c>
+      <c r="M7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" t="s">
+        <v>54</v>
+      </c>
+      <c r="E8" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" t="s">
+        <v>55</v>
+      </c>
+      <c r="G8" t="s">
+        <v>33</v>
+      </c>
+      <c r="H8" t="s">
         <v>20</v>
-      </c>
-      <c r="K7" t="s">
-        <v>21</v>
-      </c>
-      <c r="L7">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>50</v>
-      </c>
-      <c r="B8" t="s">
-        <v>51</v>
-      </c>
-      <c r="C8" t="s">
-        <v>52</v>
-      </c>
-      <c r="D8" t="s">
-        <v>53</v>
-      </c>
-      <c r="E8" t="s">
-        <v>16</v>
-      </c>
-      <c r="F8" t="s">
-        <v>54</v>
-      </c>
-      <c r="G8" t="s">
-        <v>32</v>
-      </c>
-      <c r="H8" t="s">
-        <v>19</v>
       </c>
       <c r="I8">
         <v>462.92</v>
       </c>
       <c r="J8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L8">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+      <c r="M8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I9">
         <v>530.25</v>
       </c>
       <c r="J9" t="s">
+        <v>21</v>
+      </c>
+      <c r="K9" t="s">
+        <v>22</v>
+      </c>
+      <c r="L9">
+        <v>59</v>
+      </c>
+      <c r="M9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" t="s">
+        <v>59</v>
+      </c>
+      <c r="D10" t="s">
+        <v>37</v>
+      </c>
+      <c r="E10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F10" t="s">
+        <v>55</v>
+      </c>
+      <c r="G10" t="s">
+        <v>33</v>
+      </c>
+      <c r="H10" t="s">
         <v>20</v>
-      </c>
-      <c r="K9" t="s">
-        <v>21</v>
-      </c>
-      <c r="L9">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>57</v>
-      </c>
-      <c r="B10" t="s">
-        <v>23</v>
-      </c>
-      <c r="C10" t="s">
-        <v>58</v>
-      </c>
-      <c r="D10" t="s">
-        <v>36</v>
-      </c>
-      <c r="E10" t="s">
-        <v>25</v>
-      </c>
-      <c r="F10" t="s">
-        <v>54</v>
-      </c>
-      <c r="G10" t="s">
-        <v>32</v>
-      </c>
-      <c r="H10" t="s">
-        <v>19</v>
       </c>
       <c r="I10">
         <v>335.04</v>
       </c>
       <c r="J10" t="s">
+        <v>21</v>
+      </c>
+      <c r="K10" t="s">
+        <v>22</v>
+      </c>
+      <c r="L10">
+        <v>60</v>
+      </c>
+      <c r="M10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>60</v>
+      </c>
+      <c r="B11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" t="s">
+        <v>61</v>
+      </c>
+      <c r="D11" t="s">
+        <v>54</v>
+      </c>
+      <c r="E11" t="s">
+        <v>26</v>
+      </c>
+      <c r="F11" t="s">
+        <v>32</v>
+      </c>
+      <c r="G11" t="s">
+        <v>33</v>
+      </c>
+      <c r="H11" t="s">
         <v>20</v>
-      </c>
-      <c r="K10" t="s">
-        <v>21</v>
-      </c>
-      <c r="L10">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>59</v>
-      </c>
-      <c r="B11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" t="s">
-        <v>60</v>
-      </c>
-      <c r="D11" t="s">
-        <v>53</v>
-      </c>
-      <c r="E11" t="s">
-        <v>25</v>
-      </c>
-      <c r="F11" t="s">
-        <v>31</v>
-      </c>
-      <c r="G11" t="s">
-        <v>32</v>
-      </c>
-      <c r="H11" t="s">
-        <v>19</v>
       </c>
       <c r="I11">
         <v>291.51</v>
       </c>
       <c r="J11" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K11" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L11">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+        <v>81</v>
+      </c>
+      <c r="M11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D12" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F12" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G12" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I12">
         <v>454.29</v>
       </c>
       <c r="J12" t="s">
+        <v>21</v>
+      </c>
+      <c r="K12" t="s">
+        <v>22</v>
+      </c>
+      <c r="L12">
+        <v>82</v>
+      </c>
+      <c r="M12" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>64</v>
+      </c>
+      <c r="B13" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" t="s">
+        <v>65</v>
+      </c>
+      <c r="D13" t="s">
+        <v>47</v>
+      </c>
+      <c r="E13" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" t="s">
+        <v>55</v>
+      </c>
+      <c r="G13" t="s">
+        <v>66</v>
+      </c>
+      <c r="H13" t="s">
         <v>20</v>
-      </c>
-      <c r="K12" t="s">
-        <v>21</v>
-      </c>
-      <c r="L12">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>63</v>
-      </c>
-      <c r="B13" t="s">
-        <v>44</v>
-      </c>
-      <c r="C13" t="s">
-        <v>64</v>
-      </c>
-      <c r="D13" t="s">
-        <v>46</v>
-      </c>
-      <c r="E13" t="s">
-        <v>25</v>
-      </c>
-      <c r="F13" t="s">
-        <v>54</v>
-      </c>
-      <c r="G13" t="s">
-        <v>65</v>
-      </c>
-      <c r="H13" t="s">
-        <v>19</v>
       </c>
       <c r="I13">
         <v>244.68</v>
       </c>
       <c r="J13" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K13" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L13">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+        <v>83</v>
+      </c>
+      <c r="M13" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B14" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C14" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G14" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H14" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I14">
         <v>495.44</v>
       </c>
       <c r="J14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K14" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L14">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+        <v>84</v>
+      </c>
+      <c r="M14" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B15" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D15" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E15" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F15" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G15" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I15">
         <v>513.75</v>
       </c>
       <c r="J15" t="s">
+        <v>21</v>
+      </c>
+      <c r="K15" t="s">
+        <v>22</v>
+      </c>
+      <c r="L15">
+        <v>85</v>
+      </c>
+      <c r="M15" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>71</v>
+      </c>
+      <c r="B16" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" t="s">
+        <v>72</v>
+      </c>
+      <c r="D16" t="s">
+        <v>31</v>
+      </c>
+      <c r="E16" t="s">
+        <v>26</v>
+      </c>
+      <c r="F16" t="s">
+        <v>55</v>
+      </c>
+      <c r="G16" t="s">
+        <v>73</v>
+      </c>
+      <c r="H16" t="s">
         <v>20</v>
-      </c>
-      <c r="K15" t="s">
-        <v>21</v>
-      </c>
-      <c r="L15">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>70</v>
-      </c>
-      <c r="B16" t="s">
-        <v>23</v>
-      </c>
-      <c r="C16" t="s">
-        <v>71</v>
-      </c>
-      <c r="D16" t="s">
-        <v>30</v>
-      </c>
-      <c r="E16" t="s">
-        <v>25</v>
-      </c>
-      <c r="F16" t="s">
-        <v>54</v>
-      </c>
-      <c r="G16" t="s">
-        <v>72</v>
-      </c>
-      <c r="H16" t="s">
-        <v>19</v>
       </c>
       <c r="I16">
         <v>334.98</v>
       </c>
       <c r="J16" t="s">
+        <v>21</v>
+      </c>
+      <c r="K16" t="s">
+        <v>22</v>
+      </c>
+      <c r="L16">
+        <v>86</v>
+      </c>
+      <c r="M16" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>74</v>
+      </c>
+      <c r="B17" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" t="s">
+        <v>75</v>
+      </c>
+      <c r="D17" t="s">
+        <v>31</v>
+      </c>
+      <c r="E17" t="s">
+        <v>26</v>
+      </c>
+      <c r="F17" t="s">
+        <v>55</v>
+      </c>
+      <c r="G17" t="s">
+        <v>76</v>
+      </c>
+      <c r="H17" t="s">
         <v>20</v>
-      </c>
-      <c r="K16" t="s">
-        <v>21</v>
-      </c>
-      <c r="L16">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>73</v>
-      </c>
-      <c r="B17" t="s">
-        <v>28</v>
-      </c>
-      <c r="C17" t="s">
-        <v>74</v>
-      </c>
-      <c r="D17" t="s">
-        <v>30</v>
-      </c>
-      <c r="E17" t="s">
-        <v>25</v>
-      </c>
-      <c r="F17" t="s">
-        <v>54</v>
-      </c>
-      <c r="G17" t="s">
-        <v>75</v>
-      </c>
-      <c r="H17" t="s">
-        <v>19</v>
       </c>
       <c r="I17">
         <v>234.05</v>
       </c>
       <c r="J17" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K17" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L17">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+        <v>87</v>
+      </c>
+      <c r="M17" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B18" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D18" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F18" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G18" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H18" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I18">
         <v>212.63</v>
       </c>
       <c r="J18" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K18" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L18">
+        <v>88</v>
+      </c>
+      <c r="M18" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>80</v>
+      </c>
+      <c r="B19" t="s">
+        <v>35</v>
+      </c>
+      <c r="C19" t="s">
+        <v>81</v>
+      </c>
+      <c r="D19" t="s">
+        <v>31</v>
+      </c>
+      <c r="E19" t="s">
+        <v>26</v>
+      </c>
+      <c r="F19" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>79</v>
-      </c>
-      <c r="B19" t="s">
-        <v>34</v>
-      </c>
-      <c r="C19" t="s">
-        <v>80</v>
-      </c>
-      <c r="D19" t="s">
-        <v>30</v>
-      </c>
-      <c r="E19" t="s">
-        <v>25</v>
-      </c>
-      <c r="F19" t="s">
-        <v>54</v>
-      </c>
       <c r="G19" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H19" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I19">
         <v>276.06</v>
       </c>
       <c r="J19" t="s">
+        <v>21</v>
+      </c>
+      <c r="K19" t="s">
+        <v>22</v>
+      </c>
+      <c r="L19">
+        <v>89</v>
+      </c>
+      <c r="M19" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>82</v>
+      </c>
+      <c r="B20" t="s">
+        <v>41</v>
+      </c>
+      <c r="C20" t="s">
+        <v>83</v>
+      </c>
+      <c r="D20" t="s">
+        <v>54</v>
+      </c>
+      <c r="E20" t="s">
+        <v>17</v>
+      </c>
+      <c r="F20" t="s">
+        <v>32</v>
+      </c>
+      <c r="G20" t="s">
+        <v>76</v>
+      </c>
+      <c r="H20" t="s">
         <v>20</v>
-      </c>
-      <c r="K19" t="s">
-        <v>21</v>
-      </c>
-      <c r="L19">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>81</v>
-      </c>
-      <c r="B20" t="s">
-        <v>40</v>
-      </c>
-      <c r="C20" t="s">
-        <v>82</v>
-      </c>
-      <c r="D20" t="s">
-        <v>53</v>
-      </c>
-      <c r="E20" t="s">
-        <v>16</v>
-      </c>
-      <c r="F20" t="s">
-        <v>31</v>
-      </c>
-      <c r="G20" t="s">
-        <v>75</v>
-      </c>
-      <c r="H20" t="s">
-        <v>19</v>
       </c>
       <c r="I20">
         <v>430.1</v>
       </c>
       <c r="J20" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K20" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L20">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+        <v>90</v>
+      </c>
+      <c r="M20" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B21" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C21" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D21" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E21" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F21" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G21" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H21" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I21">
         <v>255.03</v>
       </c>
       <c r="J21" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K21" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L21">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+        <v>91</v>
+      </c>
+      <c r="M21" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B22" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C22" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D22" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E22" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F22" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G22" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H22" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I22">
         <v>525.97</v>
       </c>
       <c r="J22" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K22" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L22">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+      <c r="M22" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B23" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C23" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D23" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E23" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F23" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G23" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H23" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I23">
         <v>320.67</v>
       </c>
       <c r="J23" t="s">
+        <v>21</v>
+      </c>
+      <c r="K23" t="s">
+        <v>22</v>
+      </c>
+      <c r="L23">
+        <v>94</v>
+      </c>
+      <c r="M23" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>90</v>
+      </c>
+      <c r="B24" t="s">
+        <v>29</v>
+      </c>
+      <c r="C24" t="s">
+        <v>91</v>
+      </c>
+      <c r="D24" t="s">
+        <v>54</v>
+      </c>
+      <c r="E24" t="s">
+        <v>26</v>
+      </c>
+      <c r="F24" t="s">
+        <v>48</v>
+      </c>
+      <c r="G24" t="s">
+        <v>38</v>
+      </c>
+      <c r="H24" t="s">
         <v>20</v>
-      </c>
-      <c r="K23" t="s">
-        <v>21</v>
-      </c>
-      <c r="L23">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>89</v>
-      </c>
-      <c r="B24" t="s">
-        <v>28</v>
-      </c>
-      <c r="C24" t="s">
-        <v>90</v>
-      </c>
-      <c r="D24" t="s">
-        <v>53</v>
-      </c>
-      <c r="E24" t="s">
-        <v>25</v>
-      </c>
-      <c r="F24" t="s">
-        <v>47</v>
-      </c>
-      <c r="G24" t="s">
-        <v>37</v>
-      </c>
-      <c r="H24" t="s">
-        <v>19</v>
       </c>
       <c r="I24">
         <v>232.79</v>
       </c>
       <c r="J24" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K24" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L24">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+        <v>95</v>
+      </c>
+      <c r="M24" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B25" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C25" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D25" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E25" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F25" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G25" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H25" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I25">
         <v>187.57</v>
       </c>
       <c r="J25" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K25" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L25">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+      <c r="M25" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B26" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C26" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D26" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E26" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F26" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G26" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H26" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I26">
         <v>282.32</v>
       </c>
       <c r="J26" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K26" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L26">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+        <v>97</v>
+      </c>
+      <c r="M26" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B27" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C27" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D27" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E27" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F27" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G27" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H27" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I27">
         <v>414.63</v>
       </c>
       <c r="J27" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K27" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L27">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+        <v>98</v>
+      </c>
+      <c r="M27" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B28" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C28" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D28" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E28" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F28" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G28" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H28" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I28">
         <v>259.47</v>
       </c>
       <c r="J28" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K28" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L28">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+      <c r="M28" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B29" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C29" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D29" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E29" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F29" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G29" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H29" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I29">
         <v>496.52</v>
       </c>
       <c r="J29" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K29" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L29">
-        <v>67</v>
+        <v>100</v>
+      </c>
+      <c r="M29" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
+  <autoFilter ref="A1:M1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -1856,17 +1946,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="10" width="14" customWidth="1"/>
     <col min="11" max="11" width="30" customWidth="1"/>
-    <col min="12" max="12" width="14" customWidth="1"/>
+    <col min="12" max="13" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1903,389 +1993,422 @@
       <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M1" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I2">
         <v>209.91</v>
       </c>
       <c r="J2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L2">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+      <c r="M2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I3">
         <v>201.45</v>
       </c>
       <c r="J3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L3">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+      <c r="M3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I4">
         <v>493.73</v>
       </c>
       <c r="J4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L4">
+        <v>64</v>
+      </c>
+      <c r="M4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>106</v>
+      </c>
+      <c r="B5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>105</v>
-      </c>
-      <c r="B5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" t="s">
-        <v>30</v>
-      </c>
       <c r="E5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I5">
         <v>487.74</v>
       </c>
       <c r="J5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L5">
+        <v>66</v>
+      </c>
+      <c r="M5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>107</v>
+      </c>
+      <c r="B6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E6" t="s">
+        <v>79</v>
+      </c>
+      <c r="F6" t="s">
+        <v>32</v>
+      </c>
+      <c r="G6" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>106</v>
-      </c>
-      <c r="B6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" t="s">
-        <v>30</v>
-      </c>
-      <c r="E6" t="s">
-        <v>78</v>
-      </c>
-      <c r="F6" t="s">
-        <v>31</v>
-      </c>
-      <c r="G6" t="s">
-        <v>32</v>
-      </c>
       <c r="H6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I6">
         <v>190.06</v>
       </c>
       <c r="J6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L6">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+      <c r="M6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I7">
         <v>208.52</v>
       </c>
       <c r="J7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L7">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+      <c r="M7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I8">
         <v>464.55</v>
       </c>
       <c r="J8" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L8">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+        <v>88</v>
+      </c>
+      <c r="M8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I9">
         <v>480.01</v>
       </c>
       <c r="J9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L9">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+        <v>90</v>
+      </c>
+      <c r="M9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F10" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I10">
         <v>470.62</v>
       </c>
       <c r="J10" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K10" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L10">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+      <c r="M10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D11" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G11" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I11">
         <v>206.45</v>
       </c>
       <c r="J11" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L11">
-        <v>67</v>
+        <v>100</v>
+      </c>
+      <c r="M11" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
+  <autoFilter ref="A1:M1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>